<commit_message>
updast cases and rtm
</commit_message>
<xml_diff>
--- a/OpenCart-BugReports.xlsx
+++ b/OpenCart-BugReports.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/15d74eb5e75247de/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/15d74eb5e75247de/Desktop/SQA_Projects/ManualTesting_OpenCart/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{1A17F5C7-22CC-4C2E-A35B-CC0805318596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CC127803-6F3A-4ABB-9129-956E6C68B20B}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{1A17F5C7-22CC-4C2E-A35B-CC0805318596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D06A33F6-AA7C-41D5-976E-E4019DB5D76D}"/>
   <bookViews>
-    <workbookView xWindow="9150" yWindow="1710" windowWidth="10080" windowHeight="7875" xr2:uid="{5848DFD0-C6C0-494D-B619-0F2440C0766E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{5848DFD0-C6C0-494D-B619-0F2440C0766E}"/>
   </bookViews>
   <sheets>
     <sheet name="Bugs" sheetId="1" r:id="rId1"/>
@@ -25,14 +25,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="44">
   <si>
     <t>Bug ID</t>
   </si>
   <si>
-    <t>Expected Results</t>
-  </si>
-  <si>
     <t>Actual Result</t>
   </si>
   <si>
@@ -48,33 +45,140 @@
     <t>Priority</t>
   </si>
   <si>
-    <t>Screenshot</t>
-  </si>
-  <si>
     <t>OPENCART-BUG-1</t>
   </si>
   <si>
-    <t>Thank you for registering - email is not received to the registered email address after registering an account</t>
-  </si>
-  <si>
-    <t>1. Open the app url 
-2. Click on My Account Drop menu
-3. Select 'Register' option
-4. Enter new user valid details into the Register Account page
-5. Select the Privacy Policy checkbox option
-6. Click on Continue button</t>
-  </si>
-  <si>
-    <t>User Account should be created and an email with the subject Thank you for registering should be received by the registered email address</t>
-  </si>
-  <si>
-    <t>User Account is getting created, but the email with subject Thank you for registering is not received to the registered email address</t>
-  </si>
-  <si>
     <t>Major</t>
   </si>
   <si>
     <t>P1</t>
+  </si>
+  <si>
+    <t>Confirmed finding from the supplied workbook: registration confirmation email is not received after successful registration.</t>
+  </si>
+  <si>
+    <t>1. Open the application
+2. My Account &gt; Register
+3. Enter valid unique registration data
+4. Accept Privacy Policy
+5. Click Continue</t>
+  </si>
+  <si>
+    <t>Account is created and the registration/confirmation email is received at the registered address.</t>
+  </si>
+  <si>
+    <t>Account is created, but the expected registration email was not received.</t>
+  </si>
+  <si>
+    <t>Confirmed from supplied testing work</t>
+  </si>
+  <si>
+    <t>OPENCART-BUG-2</t>
+  </si>
+  <si>
+    <t>[VERIFY] Cart total may not update correctly after changing item quantity without refreshing.</t>
+  </si>
+  <si>
+    <t>1. Add a product to cart
+2. Open Shopping Cart
+3. Change quantity from 1 to 2
+4. Click Update
+5. Compare subtotal/total with unit price × quantity</t>
+  </si>
+  <si>
+    <t>Subtotal and total should immediately reflect the updated quantity.</t>
+  </si>
+  <si>
+    <t>Record the observed result after execution; do not mark as a defect until reproduced.</t>
+  </si>
+  <si>
+    <t>Candidate — execute and verify</t>
+  </si>
+  <si>
+    <t>OPENCART-BUG-3</t>
+  </si>
+  <si>
+    <t>[VERIFY] Search may return no results for a valid partial product keyword.</t>
+  </si>
+  <si>
+    <t>1. Open Search
+2. Enter a distinctive partial keyword from a known product name
+3. Submit search</t>
+  </si>
+  <si>
+    <t>Relevant matching products should be returned for the partial keyword.</t>
+  </si>
+  <si>
+    <t>Minor</t>
+  </si>
+  <si>
+    <t>P2</t>
+  </si>
+  <si>
+    <t>OPENCART-BUG-4</t>
+  </si>
+  <si>
+    <t>[VERIFY] Wishlist action may not persist the selected product for a logged-in user.</t>
+  </si>
+  <si>
+    <t>1. Log in
+2. Open a product
+3. Click Add to Wish List
+4. Open Wishlist</t>
+  </si>
+  <si>
+    <t>Selected product should appear in the wishlist.</t>
+  </si>
+  <si>
+    <t>OPENCART-BUG-5</t>
+  </si>
+  <si>
+    <t>[VERIFY] Checkout may allow progression when a required address field is empty.</t>
+  </si>
+  <si>
+    <t>1. Add product to cart
+2. Proceed to checkout
+3. Leave one required address field empty
+4. Continue</t>
+  </si>
+  <si>
+    <t>Checkout should block progression and display validation for the missing field.</t>
+  </si>
+  <si>
+    <t>OPENCART-BUG-6</t>
+  </si>
+  <si>
+    <t>[VERIFY] Account information update may display success without persisting the changed value.</t>
+  </si>
+  <si>
+    <t>1. Log in
+2. Open Account Information
+3. Change an editable field
+4. Save
+5. Reopen the page</t>
+  </si>
+  <si>
+    <t>Changed information should remain updated after reopening the page.</t>
+  </si>
+  <si>
+    <t>OPENCART-BUG-7</t>
+  </si>
+  <si>
+    <t>[VERIFY] Order History may not show the most recently completed order.</t>
+  </si>
+  <si>
+    <t>1. Complete a valid order
+2. Open My Account &gt; Order History
+3. Review the newest entry</t>
+  </si>
+  <si>
+    <t>Newest order should appear with correct order number, date, status and total.</t>
+  </si>
+  <si>
+    <t>Expected Result</t>
+  </si>
+  <si>
+    <t>Evidence</t>
   </si>
 </sst>
 </file>
@@ -90,7 +194,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -103,8 +207,19 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -112,17 +227,75 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB7B7B7"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB7B7B7"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB7B7B7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB7B7B7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB7B7B7"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB7B7B7"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFB7B7B7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -454,29 +627,29 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>6</v>
-      </c>
       <c r="H1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
+        <v>43</v>
+      </c>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
       <c r="N1" s="1"/>
@@ -492,33 +665,33 @@
       <c r="X1" s="1"/>
       <c r="Y1" s="1"/>
     </row>
-    <row r="2" spans="1:25" ht="135" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="H2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
       <c r="M2" s="1"/>
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
@@ -533,19 +706,33 @@
       <c r="X2" s="1"/>
       <c r="Y2" s="1"/>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
+    <row r="3" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J3" s="3"/>
+      <c r="K3" s="7"/>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
       <c r="O3" s="1"/>
@@ -560,19 +747,33 @@
       <c r="X3" s="1"/>
       <c r="Y3" s="1"/>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
+    <row r="4" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J4" s="3"/>
+      <c r="K4" s="7"/>
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
@@ -587,19 +788,33 @@
       <c r="X4" s="1"/>
       <c r="Y4" s="1"/>
     </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
+    <row r="5" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J5" s="3"/>
+      <c r="K5" s="7"/>
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
@@ -614,19 +829,33 @@
       <c r="X5" s="1"/>
       <c r="Y5" s="1"/>
     </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
+    <row r="6" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J6" s="3"/>
+      <c r="K6" s="7"/>
       <c r="M6" s="1"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
@@ -641,19 +870,33 @@
       <c r="X6" s="1"/>
       <c r="Y6" s="1"/>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
+    <row r="7" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J7" s="3"/>
+      <c r="K7" s="7"/>
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
@@ -668,19 +911,33 @@
       <c r="X7" s="1"/>
       <c r="Y7" s="1"/>
     </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
+    <row r="8" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J8" s="3"/>
+      <c r="K8" s="7"/>
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
@@ -699,15 +956,6 @@
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
-      <c r="K9" s="1"/>
-      <c r="L9" s="1"/>
       <c r="M9" s="1"/>
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>

</xml_diff>

<commit_message>
updated test cases and bug report
</commit_message>
<xml_diff>
--- a/OpenCart-BugReports.xlsx
+++ b/OpenCart-BugReports.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/15d74eb5e75247de/Desktop/SQA_Projects/ManualTesting_OpenCart/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{1A17F5C7-22CC-4C2E-A35B-CC0805318596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D06A33F6-AA7C-41D5-976E-E4019DB5D76D}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{1A17F5C7-22CC-4C2E-A35B-CC0805318596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9DB1B3E-DA0A-4273-82CF-485C163CD8DE}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{5848DFD0-C6C0-494D-B619-0F2440C0766E}"/>
+    <workbookView xWindow="1470" yWindow="990" windowWidth="16785" windowHeight="9300" xr2:uid="{5848DFD0-C6C0-494D-B619-0F2440C0766E}"/>
   </bookViews>
   <sheets>
     <sheet name="Bugs" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="56">
   <si>
     <t>Bug ID</t>
   </si>
@@ -48,137 +48,168 @@
     <t>OPENCART-BUG-1</t>
   </si>
   <si>
-    <t>Major</t>
-  </si>
-  <si>
     <t>P1</t>
   </si>
   <si>
-    <t>Confirmed finding from the supplied workbook: registration confirmation email is not received after successful registration.</t>
-  </si>
-  <si>
-    <t>1. Open the application
-2. My Account &gt; Register
-3. Enter valid unique registration data
-4. Accept Privacy Policy
-5. Click Continue</t>
-  </si>
-  <si>
-    <t>Account is created and the registration/confirmation email is received at the registered address.</t>
-  </si>
-  <si>
-    <t>Account is created, but the expected registration email was not received.</t>
-  </si>
-  <si>
-    <t>Confirmed from supplied testing work</t>
-  </si>
-  <si>
     <t>OPENCART-BUG-2</t>
   </si>
   <si>
-    <t>[VERIFY] Cart total may not update correctly after changing item quantity without refreshing.</t>
-  </si>
-  <si>
-    <t>1. Add a product to cart
+    <t>OPENCART-BUG-3</t>
+  </si>
+  <si>
+    <t>P2</t>
+  </si>
+  <si>
+    <t>OPENCART-BUG-4</t>
+  </si>
+  <si>
+    <t>OPENCART-BUG-5</t>
+  </si>
+  <si>
+    <t>OPENCART-BUG-6</t>
+  </si>
+  <si>
+    <t>Expected Result</t>
+  </si>
+  <si>
+    <t>Evidence</t>
+  </si>
+  <si>
+    <t>TC_019</t>
+  </si>
+  <si>
+    <t>Test Case ID</t>
+  </si>
+  <si>
+    <t>TC_023</t>
+  </si>
+  <si>
+    <t>TC_024</t>
+  </si>
+  <si>
+    <t>TC_025</t>
+  </si>
+  <si>
+    <t>TC_035</t>
+  </si>
+  <si>
+    <t>Defect Type</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Bug Title</t>
+  </si>
+  <si>
+    <t>Shopping cart quantity x Unit Price and Subtotal calculations incorrect</t>
+  </si>
+  <si>
+    <t>Checkout button does not proceed to checkout confirmation flow</t>
+  </si>
+  <si>
+    <t>Account information update suceeds without displaying confirmation message</t>
+  </si>
+  <si>
+    <t>Password change succeeds without displaying confirmation message</t>
+  </si>
+  <si>
+    <t>Newsletter preference update suceeds without displaying confirmation message</t>
+  </si>
+  <si>
+    <t>The cart does not calculate the amount and subtotal correctly from displayed quantity and unit price</t>
+  </si>
+  <si>
+    <t>Selecting Checkout from the shopping Cart does not navigate the user to the next checkout step</t>
+  </si>
+  <si>
+    <t>Account information is saved but the expected success confirmation is not displayed</t>
+  </si>
+  <si>
+    <t>The password change is completed but the expected success confirmation is not displayed</t>
+  </si>
+  <si>
+    <t>Newsletter preference is saved but the expected success confirmation is not displayed</t>
+  </si>
+  <si>
+    <t>1. Add two or more products to cart 
 2. Open Shopping Cart
-3. Change quantity from 1 to 2
-4. Click Update
-5. Compare subtotal/total with unit price × quantity</t>
-  </si>
-  <si>
-    <t>Subtotal and total should immediately reflect the updated quantity.</t>
-  </si>
-  <si>
-    <t>Record the observed result after execution; do not mark as a defect until reproduced.</t>
-  </si>
-  <si>
-    <t>Candidate — execute and verify</t>
-  </si>
-  <si>
-    <t>OPENCART-BUG-3</t>
-  </si>
-  <si>
-    <t>[VERIFY] Search may return no results for a valid partial product keyword.</t>
-  </si>
-  <si>
-    <t>1. Open Search
-2. Enter a distinctive partial keyword from a known product name
-3. Submit search</t>
-  </si>
-  <si>
-    <t>Relevant matching products should be returned for the partial keyword.</t>
-  </si>
-  <si>
-    <t>Minor</t>
-  </si>
-  <si>
-    <t>P2</t>
-  </si>
-  <si>
-    <t>OPENCART-BUG-4</t>
-  </si>
-  <si>
-    <t>[VERIFY] Wishlist action may not persist the selected product for a logged-in user.</t>
+3. Calculate expected Quantity x Unit price and Subtotal
+4. Compare with displayed values</t>
+  </si>
+  <si>
+    <t>1. Add a product to the cart
+2. Open Shopping Cart
+3. Click checkout
+4. Observe the page
+5. The first checkout order works but the second time a new check out order does not work</t>
+  </si>
+  <si>
+    <t>1. Login
+2. Open My Account&gt;Edit your account information
+3. Change an editable field 
+4. Click Continue
+5. Observe the resultig page/ message</t>
   </si>
   <si>
     <t>1. Log in
-2. Open a product
-3. Click Add to Wish List
-4. Open Wishlist</t>
-  </si>
-  <si>
-    <t>Selected product should appear in the wishlist.</t>
-  </si>
-  <si>
-    <t>OPENCART-BUG-5</t>
-  </si>
-  <si>
-    <t>[VERIFY] Checkout may allow progression when a required address field is empty.</t>
-  </si>
-  <si>
-    <t>1. Add product to cart
-2. Proceed to checkout
-3. Leave one required address field empty
-4. Continue</t>
-  </si>
-  <si>
-    <t>Checkout should block progression and display validation for the missing field.</t>
-  </si>
-  <si>
-    <t>OPENCART-BUG-6</t>
-  </si>
-  <si>
-    <t>[VERIFY] Account information update may display success without persisting the changed value.</t>
-  </si>
-  <si>
-    <t>1. Log in
-2. Open Account Information
-3. Change an editable field
-4. Save
-5. Reopen the page</t>
-  </si>
-  <si>
-    <t>Changed information should remain updated after reopening the page.</t>
-  </si>
-  <si>
-    <t>OPENCART-BUG-7</t>
-  </si>
-  <si>
-    <t>[VERIFY] Order History may not show the most recently completed order.</t>
-  </si>
-  <si>
-    <t>1. Complete a valid order
-2. Open My Account &gt; Order History
-3. Review the newest entry</t>
-  </si>
-  <si>
-    <t>Newest order should appear with correct order number, date, status and total.</t>
-  </si>
-  <si>
-    <t>Expected Result</t>
-  </si>
-  <si>
-    <t>Evidence</t>
+2. Open My Account&gt; Change Password
+3. Enter current password and matching new password and Save
+4. Observe the resulting page/ message</t>
+  </si>
+  <si>
+    <t>1. Login
+2. Open My Account &gt; Newsletter
+3. Change Newsletter preference and Save/ Continue
+4. Observe the resulting page/ message</t>
+  </si>
+  <si>
+    <t>Line amount should be calculated correctly from quantity, unit price and applicable charges</t>
+  </si>
+  <si>
+    <t>The application should navigate to the checkout flow so the user can select/ confirm shipping and complete the order</t>
+  </si>
+  <si>
+    <t>Updated information is saved and a confirmation/success message is displayed</t>
+  </si>
+  <si>
+    <t>Password is changed successfully and a confirmation/ success message is displayed</t>
+  </si>
+  <si>
+    <t>Newsletter preference is saved and a confirmation/ success message is displayed</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Quantity x Unit Price calculation wrong and Subtotal calculation is wrong</t>
+  </si>
+  <si>
+    <t>It remains  on the Shopping Cart page and does not redirect to the next checkout step</t>
+  </si>
+  <si>
+    <t>Update is saved and the user is redirected to My Account but no confirmation is displayed</t>
+  </si>
+  <si>
+    <t>Password is changed successfully but no confirmation message displayed</t>
+  </si>
+  <si>
+    <t>Newsletter preference is saved and the user is redirected to My Account but no confirmation is displayed</t>
+  </si>
+  <si>
+    <t>Calculation/ Functional</t>
+  </si>
+  <si>
+    <t>Navigation/ Functional</t>
+  </si>
+  <si>
+    <t>UI/ Feedback</t>
+  </si>
+  <si>
+    <t>New</t>
   </si>
 </sst>
 </file>
@@ -194,7 +225,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -205,11 +236,6 @@
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9EAF7"/>
       </patternFill>
     </fill>
     <fill>
@@ -285,18 +311,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -611,49 +635,58 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{687C089C-C374-431F-A8D3-88EA4DF56063}">
-  <dimension ref="A1:Y40"/>
+  <dimension ref="A1:AC40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" customWidth="1"/>
-    <col min="2" max="2" width="27.7109375" customWidth="1"/>
-    <col min="3" max="3" width="30.7109375" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" customWidth="1"/>
-    <col min="5" max="5" width="17.140625" customWidth="1"/>
-    <col min="8" max="8" width="16.140625" customWidth="1"/>
+    <col min="1" max="3" width="17.42578125" customWidth="1"/>
+    <col min="4" max="4" width="27.7109375" customWidth="1"/>
+    <col min="5" max="5" width="30.7109375" customWidth="1"/>
+    <col min="6" max="6" width="28.85546875" customWidth="1"/>
+    <col min="7" max="7" width="17.140625" customWidth="1"/>
+    <col min="10" max="11" width="12.42578125" customWidth="1"/>
+    <col min="12" max="12" width="16.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
+      <c r="J1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="M1" s="5"/>
+      <c r="N1" s="5"/>
+      <c r="O1" s="5"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -664,38 +697,48 @@
       <c r="W1" s="1"/>
       <c r="X1" s="1"/>
       <c r="Y1" s="1"/>
-    </row>
-    <row r="2" spans="1:25" ht="90" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
+    </row>
+    <row r="2" spans="1:29" ht="105" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="F2" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="I2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
+      <c r="J2" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="L2" s="3"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
       <c r="S2" s="1"/>
@@ -705,38 +748,48 @@
       <c r="W2" s="1"/>
       <c r="X2" s="1"/>
       <c r="Y2" s="1"/>
-    </row>
-    <row r="3" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+      <c r="Z2" s="1"/>
+      <c r="AA2" s="1"/>
+      <c r="AB2" s="1"/>
+      <c r="AC2" s="1"/>
+    </row>
+    <row r="3" spans="1:29" ht="105" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="F3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="I3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="J3" s="3"/>
-      <c r="K3" s="7"/>
-      <c r="M3" s="1"/>
-      <c r="N3" s="1"/>
-      <c r="O3" s="1"/>
-      <c r="P3" s="1"/>
+      <c r="J3" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="L3" s="6"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="6"/>
       <c r="Q3" s="1"/>
       <c r="R3" s="1"/>
       <c r="S3" s="1"/>
@@ -746,38 +799,48 @@
       <c r="W3" s="1"/>
       <c r="X3" s="1"/>
       <c r="Y3" s="1"/>
-    </row>
-    <row r="4" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+      <c r="Z3" s="1"/>
+      <c r="AA3" s="1"/>
+      <c r="AB3" s="1"/>
+      <c r="AC3" s="1"/>
+    </row>
+    <row r="4" spans="1:29" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="J4" s="3"/>
-      <c r="K4" s="7"/>
-      <c r="M4" s="1"/>
-      <c r="N4" s="1"/>
-      <c r="O4" s="1"/>
-      <c r="P4" s="1"/>
+        <v>49</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="L4" s="6"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="6"/>
       <c r="Q4" s="1"/>
       <c r="R4" s="1"/>
       <c r="S4" s="1"/>
@@ -787,38 +850,48 @@
       <c r="W4" s="1"/>
       <c r="X4" s="1"/>
       <c r="Y4" s="1"/>
-    </row>
-    <row r="5" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+      <c r="Z4" s="1"/>
+      <c r="AA4" s="1"/>
+      <c r="AB4" s="1"/>
+      <c r="AC4" s="1"/>
+    </row>
+    <row r="5" spans="1:29" ht="120" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>28</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>7</v>
+        <v>43</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="J5" s="3"/>
-      <c r="K5" s="7"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
-      <c r="P5" s="1"/>
+        <v>50</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="L5" s="6"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="6"/>
       <c r="Q5" s="1"/>
       <c r="R5" s="1"/>
       <c r="S5" s="1"/>
@@ -828,38 +901,48 @@
       <c r="W5" s="1"/>
       <c r="X5" s="1"/>
       <c r="Y5" s="1"/>
-    </row>
-    <row r="6" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+      <c r="Z5" s="1"/>
+      <c r="AA5" s="1"/>
+      <c r="AB5" s="1"/>
+      <c r="AC5" s="1"/>
+    </row>
+    <row r="6" spans="1:29" ht="105" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="J6" s="3"/>
-      <c r="K6" s="7"/>
-      <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
-      <c r="O6" s="1"/>
-      <c r="P6" s="1"/>
+        <v>51</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="L6" s="6"/>
+      <c r="N6" s="3"/>
+      <c r="O6" s="6"/>
       <c r="Q6" s="1"/>
       <c r="R6" s="1"/>
       <c r="S6" s="1"/>
@@ -869,38 +952,28 @@
       <c r="W6" s="1"/>
       <c r="X6" s="1"/>
       <c r="Y6" s="1"/>
-    </row>
-    <row r="7" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+      <c r="Z6" s="1"/>
+      <c r="AA6" s="1"/>
+      <c r="AB6" s="1"/>
+      <c r="AC6" s="1"/>
+    </row>
+    <row r="7" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>19</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
       <c r="J7" s="3"/>
-      <c r="K7" s="7"/>
-      <c r="M7" s="1"/>
-      <c r="N7" s="1"/>
-      <c r="O7" s="1"/>
-      <c r="P7" s="1"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="6"/>
+      <c r="N7" s="3"/>
+      <c r="O7" s="6"/>
       <c r="Q7" s="1"/>
       <c r="R7" s="1"/>
       <c r="S7" s="1"/>
@@ -910,38 +983,25 @@
       <c r="W7" s="1"/>
       <c r="X7" s="1"/>
       <c r="Y7" s="1"/>
-    </row>
-    <row r="8" spans="1:25" ht="90" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>19</v>
-      </c>
+      <c r="Z7" s="1"/>
+      <c r="AA7" s="1"/>
+      <c r="AB7" s="1"/>
+      <c r="AC7" s="1"/>
+    </row>
+    <row r="8" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
       <c r="J8" s="3"/>
-      <c r="K8" s="7"/>
-      <c r="M8" s="1"/>
-      <c r="N8" s="1"/>
-      <c r="O8" s="1"/>
-      <c r="P8" s="1"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="6"/>
+      <c r="N8" s="3"/>
+      <c r="O8" s="6"/>
       <c r="Q8" s="1"/>
       <c r="R8" s="1"/>
       <c r="S8" s="1"/>
@@ -951,15 +1011,16 @@
       <c r="W8" s="1"/>
       <c r="X8" s="1"/>
       <c r="Y8" s="1"/>
-    </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A9" s="1"/>
+      <c r="Z8" s="1"/>
+      <c r="AA8" s="1"/>
+      <c r="AB8" s="1"/>
+      <c r="AC8" s="1"/>
+    </row>
+    <row r="9" spans="1:29" x14ac:dyDescent="0.25">
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
-      <c r="M9" s="1"/>
-      <c r="N9" s="1"/>
-      <c r="O9" s="1"/>
-      <c r="P9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
       <c r="Q9" s="1"/>
       <c r="R9" s="1"/>
       <c r="S9" s="1"/>
@@ -969,9 +1030,12 @@
       <c r="W9" s="1"/>
       <c r="X9" s="1"/>
       <c r="Y9" s="1"/>
-    </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A10" s="1"/>
+      <c r="Z9" s="1"/>
+      <c r="AA9" s="1"/>
+      <c r="AB9" s="1"/>
+      <c r="AC9" s="1"/>
+    </row>
+    <row r="10" spans="1:29" x14ac:dyDescent="0.25">
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -996,9 +1060,12 @@
       <c r="W10" s="1"/>
       <c r="X10" s="1"/>
       <c r="Y10" s="1"/>
-    </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A11" s="1"/>
+      <c r="Z10" s="1"/>
+      <c r="AA10" s="1"/>
+      <c r="AB10" s="1"/>
+      <c r="AC10" s="1"/>
+    </row>
+    <row r="11" spans="1:29" x14ac:dyDescent="0.25">
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
@@ -1023,9 +1090,12 @@
       <c r="W11" s="1"/>
       <c r="X11" s="1"/>
       <c r="Y11" s="1"/>
-    </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A12" s="1"/>
+      <c r="Z11" s="1"/>
+      <c r="AA11" s="1"/>
+      <c r="AB11" s="1"/>
+      <c r="AC11" s="1"/>
+    </row>
+    <row r="12" spans="1:29" x14ac:dyDescent="0.25">
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
@@ -1050,9 +1120,12 @@
       <c r="W12" s="1"/>
       <c r="X12" s="1"/>
       <c r="Y12" s="1"/>
-    </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A13" s="1"/>
+      <c r="Z12" s="1"/>
+      <c r="AA12" s="1"/>
+      <c r="AB12" s="1"/>
+      <c r="AC12" s="1"/>
+    </row>
+    <row r="13" spans="1:29" x14ac:dyDescent="0.25">
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
@@ -1077,9 +1150,12 @@
       <c r="W13" s="1"/>
       <c r="X13" s="1"/>
       <c r="Y13" s="1"/>
-    </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A14" s="1"/>
+      <c r="Z13" s="1"/>
+      <c r="AA13" s="1"/>
+      <c r="AB13" s="1"/>
+      <c r="AC13" s="1"/>
+    </row>
+    <row r="14" spans="1:29" x14ac:dyDescent="0.25">
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
@@ -1104,9 +1180,12 @@
       <c r="W14" s="1"/>
       <c r="X14" s="1"/>
       <c r="Y14" s="1"/>
-    </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A15" s="1"/>
+      <c r="Z14" s="1"/>
+      <c r="AA14" s="1"/>
+      <c r="AB14" s="1"/>
+      <c r="AC14" s="1"/>
+    </row>
+    <row r="15" spans="1:29" x14ac:dyDescent="0.25">
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
@@ -1131,9 +1210,12 @@
       <c r="W15" s="1"/>
       <c r="X15" s="1"/>
       <c r="Y15" s="1"/>
-    </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A16" s="1"/>
+      <c r="Z15" s="1"/>
+      <c r="AA15" s="1"/>
+      <c r="AB15" s="1"/>
+      <c r="AC15" s="1"/>
+    </row>
+    <row r="16" spans="1:29" x14ac:dyDescent="0.25">
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
@@ -1158,9 +1240,12 @@
       <c r="W16" s="1"/>
       <c r="X16" s="1"/>
       <c r="Y16" s="1"/>
-    </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A17" s="1"/>
+      <c r="Z16" s="1"/>
+      <c r="AA16" s="1"/>
+      <c r="AB16" s="1"/>
+      <c r="AC16" s="1"/>
+    </row>
+    <row r="17" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
@@ -1185,9 +1270,12 @@
       <c r="W17" s="1"/>
       <c r="X17" s="1"/>
       <c r="Y17" s="1"/>
-    </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A18" s="1"/>
+      <c r="Z17" s="1"/>
+      <c r="AA17" s="1"/>
+      <c r="AB17" s="1"/>
+      <c r="AC17" s="1"/>
+    </row>
+    <row r="18" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
@@ -1212,9 +1300,12 @@
       <c r="W18" s="1"/>
       <c r="X18" s="1"/>
       <c r="Y18" s="1"/>
-    </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A19" s="1"/>
+      <c r="Z18" s="1"/>
+      <c r="AA18" s="1"/>
+      <c r="AB18" s="1"/>
+      <c r="AC18" s="1"/>
+    </row>
+    <row r="19" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
@@ -1239,9 +1330,12 @@
       <c r="W19" s="1"/>
       <c r="X19" s="1"/>
       <c r="Y19" s="1"/>
-    </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A20" s="1"/>
+      <c r="Z19" s="1"/>
+      <c r="AA19" s="1"/>
+      <c r="AB19" s="1"/>
+      <c r="AC19" s="1"/>
+    </row>
+    <row r="20" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
@@ -1266,9 +1360,12 @@
       <c r="W20" s="1"/>
       <c r="X20" s="1"/>
       <c r="Y20" s="1"/>
-    </row>
-    <row r="21" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A21" s="1"/>
+      <c r="Z20" s="1"/>
+      <c r="AA20" s="1"/>
+      <c r="AB20" s="1"/>
+      <c r="AC20" s="1"/>
+    </row>
+    <row r="21" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
@@ -1293,9 +1390,12 @@
       <c r="W21" s="1"/>
       <c r="X21" s="1"/>
       <c r="Y21" s="1"/>
-    </row>
-    <row r="22" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A22" s="1"/>
+      <c r="Z21" s="1"/>
+      <c r="AA21" s="1"/>
+      <c r="AB21" s="1"/>
+      <c r="AC21" s="1"/>
+    </row>
+    <row r="22" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
@@ -1320,9 +1420,12 @@
       <c r="W22" s="1"/>
       <c r="X22" s="1"/>
       <c r="Y22" s="1"/>
-    </row>
-    <row r="23" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A23" s="1"/>
+      <c r="Z22" s="1"/>
+      <c r="AA22" s="1"/>
+      <c r="AB22" s="1"/>
+      <c r="AC22" s="1"/>
+    </row>
+    <row r="23" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
@@ -1347,9 +1450,12 @@
       <c r="W23" s="1"/>
       <c r="X23" s="1"/>
       <c r="Y23" s="1"/>
-    </row>
-    <row r="24" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A24" s="1"/>
+      <c r="Z23" s="1"/>
+      <c r="AA23" s="1"/>
+      <c r="AB23" s="1"/>
+      <c r="AC23" s="1"/>
+    </row>
+    <row r="24" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
@@ -1374,9 +1480,12 @@
       <c r="W24" s="1"/>
       <c r="X24" s="1"/>
       <c r="Y24" s="1"/>
-    </row>
-    <row r="25" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A25" s="1"/>
+      <c r="Z24" s="1"/>
+      <c r="AA24" s="1"/>
+      <c r="AB24" s="1"/>
+      <c r="AC24" s="1"/>
+    </row>
+    <row r="25" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
@@ -1401,9 +1510,12 @@
       <c r="W25" s="1"/>
       <c r="X25" s="1"/>
       <c r="Y25" s="1"/>
-    </row>
-    <row r="26" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A26" s="1"/>
+      <c r="Z25" s="1"/>
+      <c r="AA25" s="1"/>
+      <c r="AB25" s="1"/>
+      <c r="AC25" s="1"/>
+    </row>
+    <row r="26" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
@@ -1428,9 +1540,12 @@
       <c r="W26" s="1"/>
       <c r="X26" s="1"/>
       <c r="Y26" s="1"/>
-    </row>
-    <row r="27" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A27" s="1"/>
+      <c r="Z26" s="1"/>
+      <c r="AA26" s="1"/>
+      <c r="AB26" s="1"/>
+      <c r="AC26" s="1"/>
+    </row>
+    <row r="27" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
@@ -1455,9 +1570,12 @@
       <c r="W27" s="1"/>
       <c r="X27" s="1"/>
       <c r="Y27" s="1"/>
-    </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A28" s="1"/>
+      <c r="Z27" s="1"/>
+      <c r="AA27" s="1"/>
+      <c r="AB27" s="1"/>
+      <c r="AC27" s="1"/>
+    </row>
+    <row r="28" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
@@ -1482,9 +1600,12 @@
       <c r="W28" s="1"/>
       <c r="X28" s="1"/>
       <c r="Y28" s="1"/>
-    </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A29" s="1"/>
+      <c r="Z28" s="1"/>
+      <c r="AA28" s="1"/>
+      <c r="AB28" s="1"/>
+      <c r="AC28" s="1"/>
+    </row>
+    <row r="29" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
@@ -1509,9 +1630,12 @@
       <c r="W29" s="1"/>
       <c r="X29" s="1"/>
       <c r="Y29" s="1"/>
-    </row>
-    <row r="30" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A30" s="1"/>
+      <c r="Z29" s="1"/>
+      <c r="AA29" s="1"/>
+      <c r="AB29" s="1"/>
+      <c r="AC29" s="1"/>
+    </row>
+    <row r="30" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
@@ -1536,9 +1660,12 @@
       <c r="W30" s="1"/>
       <c r="X30" s="1"/>
       <c r="Y30" s="1"/>
-    </row>
-    <row r="31" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A31" s="1"/>
+      <c r="Z30" s="1"/>
+      <c r="AA30" s="1"/>
+      <c r="AB30" s="1"/>
+      <c r="AC30" s="1"/>
+    </row>
+    <row r="31" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
@@ -1563,9 +1690,12 @@
       <c r="W31" s="1"/>
       <c r="X31" s="1"/>
       <c r="Y31" s="1"/>
-    </row>
-    <row r="32" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A32" s="1"/>
+      <c r="Z31" s="1"/>
+      <c r="AA31" s="1"/>
+      <c r="AB31" s="1"/>
+      <c r="AC31" s="1"/>
+    </row>
+    <row r="32" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
@@ -1590,9 +1720,12 @@
       <c r="W32" s="1"/>
       <c r="X32" s="1"/>
       <c r="Y32" s="1"/>
-    </row>
-    <row r="33" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A33" s="1"/>
+      <c r="Z32" s="1"/>
+      <c r="AA32" s="1"/>
+      <c r="AB32" s="1"/>
+      <c r="AC32" s="1"/>
+    </row>
+    <row r="33" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
@@ -1617,9 +1750,12 @@
       <c r="W33" s="1"/>
       <c r="X33" s="1"/>
       <c r="Y33" s="1"/>
-    </row>
-    <row r="34" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A34" s="1"/>
+      <c r="Z33" s="1"/>
+      <c r="AA33" s="1"/>
+      <c r="AB33" s="1"/>
+      <c r="AC33" s="1"/>
+    </row>
+    <row r="34" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
@@ -1644,9 +1780,12 @@
       <c r="W34" s="1"/>
       <c r="X34" s="1"/>
       <c r="Y34" s="1"/>
-    </row>
-    <row r="35" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A35" s="1"/>
+      <c r="Z34" s="1"/>
+      <c r="AA34" s="1"/>
+      <c r="AB34" s="1"/>
+      <c r="AC34" s="1"/>
+    </row>
+    <row r="35" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
@@ -1671,9 +1810,12 @@
       <c r="W35" s="1"/>
       <c r="X35" s="1"/>
       <c r="Y35" s="1"/>
-    </row>
-    <row r="36" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A36" s="1"/>
+      <c r="Z35" s="1"/>
+      <c r="AA35" s="1"/>
+      <c r="AB35" s="1"/>
+      <c r="AC35" s="1"/>
+    </row>
+    <row r="36" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
@@ -1698,9 +1840,12 @@
       <c r="W36" s="1"/>
       <c r="X36" s="1"/>
       <c r="Y36" s="1"/>
-    </row>
-    <row r="37" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A37" s="1"/>
+      <c r="Z36" s="1"/>
+      <c r="AA36" s="1"/>
+      <c r="AB36" s="1"/>
+      <c r="AC36" s="1"/>
+    </row>
+    <row r="37" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
@@ -1725,9 +1870,12 @@
       <c r="W37" s="1"/>
       <c r="X37" s="1"/>
       <c r="Y37" s="1"/>
-    </row>
-    <row r="38" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A38" s="1"/>
+      <c r="Z37" s="1"/>
+      <c r="AA37" s="1"/>
+      <c r="AB37" s="1"/>
+      <c r="AC37" s="1"/>
+    </row>
+    <row r="38" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
@@ -1752,9 +1900,12 @@
       <c r="W38" s="1"/>
       <c r="X38" s="1"/>
       <c r="Y38" s="1"/>
-    </row>
-    <row r="39" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A39" s="1"/>
+      <c r="Z38" s="1"/>
+      <c r="AA38" s="1"/>
+      <c r="AB38" s="1"/>
+      <c r="AC38" s="1"/>
+    </row>
+    <row r="39" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>
       <c r="D39" s="1"/>
@@ -1779,9 +1930,12 @@
       <c r="W39" s="1"/>
       <c r="X39" s="1"/>
       <c r="Y39" s="1"/>
-    </row>
-    <row r="40" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A40" s="1"/>
+      <c r="Z39" s="1"/>
+      <c r="AA39" s="1"/>
+      <c r="AB39" s="1"/>
+      <c r="AC39" s="1"/>
+    </row>
+    <row r="40" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
@@ -1806,6 +1960,10 @@
       <c r="W40" s="1"/>
       <c r="X40" s="1"/>
       <c r="Y40" s="1"/>
+      <c r="Z40" s="1"/>
+      <c r="AA40" s="1"/>
+      <c r="AB40" s="1"/>
+      <c r="AC40" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>